<commit_message>
Switch database connection from Oracle to Supabase PostgreSQL
</commit_message>
<xml_diff>
--- a/Card_TestCases.xlsx
+++ b/Card_TestCases.xlsx
@@ -18,12 +18,18 @@
     <sheet name="Admin _ Supervisor Functions-Ne" sheetId="11" r:id="rId14"/>
     <sheet name="Credit_Card_Positive_Scenario" sheetId="12" r:id="rId15"/>
     <sheet name="Credit_Card_Negative_Scenario" sheetId="13" r:id="rId16"/>
+    <sheet name="Other_Bank_Card_Positive_Scenar" sheetId="14" r:id="rId17"/>
+    <sheet name="Other_Bank_Card_Negative_Scenar" sheetId="15" r:id="rId18"/>
+    <sheet name="SLIC Life Positive" sheetId="16" r:id="rId19"/>
+    <sheet name="SLIC Life Negative" sheetId="17" r:id="rId20"/>
+    <sheet name="SLIC General Positive" sheetId="18" r:id="rId21"/>
+    <sheet name="SLIC General Negative" sheetId="19" r:id="rId22"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="764">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="843">
   <si>
     <t>This document was exported from Numbers. Each table was converted to an Excel worksheet. All other objects on each Numbers sheet were placed on separate worksheets. Please be aware that formula calculations may differ in Excel.</t>
   </si>
@@ -2554,6 +2560,262 @@
 2. Operation blocked.
 </t>
   </si>
+  <si>
+    <t>Other_Bank_Card_Positive_Scenario</t>
+  </si>
+  <si>
+    <t>Other_Bank_Card_Positive_Scenar</t>
+  </si>
+  <si>
+    <t>Other Bank Card Functions - Positive Scenarios</t>
+  </si>
+  <si>
+    <t>TC_CB_CW_OBC_P_01_001</t>
+  </si>
+  <si>
+    <t>Successful Cash Withdrawal (Savings)</t>
+  </si>
+  <si>
+    <t>Verify that a user can successfully withdraw cash from a Savings account using a valid card and PIN.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+1. ATM/Kiosk is online.
+2. User has a valid card, sufficient account balance, and correct PIN.
+</t>
+  </si>
+  <si>
+    <t>Transaction is approved, cash is dispensed, receipt is printed, and card is returned successfully.</t>
+  </si>
+  <si>
+    <t>TC_CB_CW_OBC_P_01_002</t>
+  </si>
+  <si>
+    <t>Successful Cash Withdrawal (Current)</t>
+  </si>
+  <si>
+    <t>Verify that a user can successfully withdraw cash from a Current account using a valid card and PIN.</t>
+  </si>
+  <si>
+    <t>1. ATM/Kiosk is online.
+2. User has a valid card, sufficient funds in Current account, and correct PIN.</t>
+  </si>
+  <si>
+    <t>Insert Card &gt; Select Language &gt; Enter valid PIN &gt; Select Withdrawal &gt; Select Current Account &gt; Enter valid amount (e.g., Rs. 10,000) &gt; Select Receipt Option &gt; Take Cash &gt; Take Receipt &amp; Card</t>
+  </si>
+  <si>
+    <t>Transaction is processed successfully, cash is dispensed, and physical/digital receipt is provided.</t>
+  </si>
+  <si>
+    <t>Other_Bank_Card_Negative_Scenario</t>
+  </si>
+  <si>
+    <t>Other_Bank_Card_Negative_Scenar</t>
+  </si>
+  <si>
+    <t>Other Bank Card Functions - Negative Scenarios</t>
+  </si>
+  <si>
+    <t>TC_CB_CW_OBC_N_01_001</t>
+  </si>
+  <si>
+    <t>Invalid PIN Entry</t>
+  </si>
+  <si>
+    <t>Verify the system response when an incorrect PIN is entered during a cash withdrawal.</t>
+  </si>
+  <si>
+    <t>1. ATM is online.
+2. User has a valid card.</t>
+  </si>
+  <si>
+    <t>Insert Card &gt; Select Language &gt; Enter invalid PIN &gt; Select Withdrawal</t>
+  </si>
+  <si>
+    <t>The system displays an incorrect PIN error message, denies access, and prompts the user to retry or retains the card after maximum attempts.</t>
+  </si>
+  <si>
+    <t>TC_CB_CW_OBC_N_01_002</t>
+  </si>
+  <si>
+    <t>Insufficient Funds</t>
+  </si>
+  <si>
+    <t>Verify that the system blocks a cash withdrawal when the requested amount exceeds the account balance.</t>
+  </si>
+  <si>
+    <t>1. ATM is online.
+2. User account has a low balance (e.g., Rs. 500).</t>
+  </si>
+  <si>
+    <t>Insert Card &gt; Select Language &gt; Enter valid PIN &gt; Select Withdrawal &gt; Select Account &gt; Enter high amount (e.g., Rs. 50,000) &gt; Confirm</t>
+  </si>
+  <si>
+    <t>The transaction is declined, an "Insufficient Funds" error message is shown, and no cash is dispensed.</t>
+  </si>
+  <si>
+    <t>TC_CB_CW_OBC_N_01_003</t>
+  </si>
+  <si>
+    <t>Exceeding Daily Withdrawal Limit</t>
+  </si>
+  <si>
+    <t>Verify the system blocks withdrawals that exceed the card's permitted daily transaction limit.</t>
+  </si>
+  <si>
+    <t>1. ATM is online.
+2. User has already reached their daily withdrawal limit.</t>
+  </si>
+  <si>
+    <t>Insert Card &gt; Select Language &gt; Enter valid PIN &gt; Select Withdrawal &gt; Select Account &gt; Enter amount exceeding limit &gt; Confirm</t>
+  </si>
+  <si>
+    <t>The transaction is rejected with a limit exceeded notification message, and no cash is dispensed.</t>
+  </si>
+  <si>
+    <t>TC_CB_CW_OBC_N_01_004</t>
+  </si>
+  <si>
+    <t>SLIC Life Positive</t>
+  </si>
+  <si>
+    <t>SLIC LIFE Functions - Positive Scenarios</t>
+  </si>
+  <si>
+    <t>TC_CB_SLIC_P_01_001</t>
+  </si>
+  <si>
+    <t>SLIC Life Insurance Payment</t>
+  </si>
+  <si>
+    <t>Verify that a user can successfully process a positive cash deposit for an SLIC Life Insurance policy using a card.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. CRM is online and functional.
+2. User has a valid card and correct PIN.
+3. Active Life Insurance customer reference number.
+</t>
+  </si>
+  <si>
+    <t>Insert Card &gt; Select Language &gt; Enter valid PIN &gt; Select Bill Payment &gt; Select SLIC &gt; Select Life Insurance &gt; Enter Customer Reference Number &gt; Enter Amount &gt; Select Account &gt; Confirm Bill Payment &gt; Take Receipt &amp; Card</t>
+  </si>
+  <si>
+    <t>Transaction is successfully processed, funds are debited/accepted, confirmation screen is shown, and receipt is printed.</t>
+  </si>
+  <si>
+    <t>SLIC Life Negative</t>
+  </si>
+  <si>
+    <t>SLIC LIFE Card Functions - Negative Scenarios</t>
+  </si>
+  <si>
+    <t>TC_CB_SLIC_N_01_001</t>
+  </si>
+  <si>
+    <t>Invalid Life Insurance Customer Ref</t>
+  </si>
+  <si>
+    <t>Verify system behavior when an invalid or non-existent SLIC Life Insurance customer reference number is entered.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. CRM is online and functional.
+2. User is authenticated with a valid card and PIN.
+</t>
+  </si>
+  <si>
+    <t>Insert Card &gt; Select Language &gt; Enter valid PIN &gt; Select Bill Payment &gt; Select SLIC &gt; Select Life Insurance &gt; Enter Invalid Customer Reference Number &gt; Enter Amount &gt; Select Account &gt; Confirm Bill Payment</t>
+  </si>
+  <si>
+    <t>System displays an error message (e.g., "Invalid Customer Reference") and blocks the transaction from completing.</t>
+  </si>
+  <si>
+    <t>TC_CB_SLIC_N_01_002</t>
+  </si>
+  <si>
+    <t>Invalid Life Insurance Amount Entry</t>
+  </si>
+  <si>
+    <t>Verify that the system rejects zero or negative amounts entered for an SLIC Life Insurance payment.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Kiosk is online and functional.
+2. User has entered a valid Life Insurance customer reference.
+</t>
+  </si>
+  <si>
+    <t>Insert Card &gt; Select Language &gt; Enter valid PIN &gt; Select Bill Payment &gt; Select SLIC &gt; Select Life Insurance &gt; Enter Customer Reference Number &gt; Enter Amount (0.00 or negative) &gt; Proceed</t>
+  </si>
+  <si>
+    <t>System blocks the transaction flow, triggers an invalid amount error message, and prompts for re-entry.</t>
+  </si>
+  <si>
+    <t>SLIC General Positive</t>
+  </si>
+  <si>
+    <t>SLIC GENERAL Functions - Positive Scenarios</t>
+  </si>
+  <si>
+    <t>TC_CB_SLIC_GEN_P_01_001</t>
+  </si>
+  <si>
+    <t>General Insurance Payment</t>
+  </si>
+  <si>
+    <t>Verify that a user can successfully process a positive cash deposit for an SLIC General Insurance policy using a card.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. CRM is online and functional.
+2. User has a valid card and correct PIN.
+3. Active General Insurance customer reference number.
+</t>
+  </si>
+  <si>
+    <t>Insert Card &gt; Select Language &gt; Enter valid PIN &gt; Select Bill Payment &gt; Select SLIC &gt; Select General Insurance &gt; Enter Customer Reference Number &gt; Enter Amount &gt; Select Account &gt; Confirm Bill Payment &gt; Take Receipt &amp; Card</t>
+  </si>
+  <si>
+    <t>Transaction is successfully processed, confirmation is displayed, and receipt containing correct General Insurance details is printed.</t>
+  </si>
+  <si>
+    <t>SLIC General Negative</t>
+  </si>
+  <si>
+    <t>SLIC GENERAL Functions - Negative Scenarios</t>
+  </si>
+  <si>
+    <t>TC_CB_SLIC_GEN_N_01_001</t>
+  </si>
+  <si>
+    <t>Invalid General Insurance Customer Ref</t>
+  </si>
+  <si>
+    <t>Verify system behavior when an invalid or non-existent SLIC General Insurance customer reference number is entered.</t>
+  </si>
+  <si>
+    <t>Insert Card &gt; Select Language &gt; Enter valid PIN &gt; Select Bill Payment &gt; Select SLIC &gt; Select General Insurance &gt; Enter Invalid Customer Reference Number &gt; Enter Amount &gt; Select Account &gt; Confirm Bill Payment</t>
+  </si>
+  <si>
+    <t>System displays an error message (e.g., "Invalid Customer Reference") and prevents proceeding to confirmation.</t>
+  </si>
+  <si>
+    <t>TC_CB_SLIC_GEN_N_01_002</t>
+  </si>
+  <si>
+    <t>Insufficient Funds for General Insurance</t>
+  </si>
+  <si>
+    <t>Verify that the transaction is declined when the selected account has insufficient funds during a General Insurance payment.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. CRM is online and functional.
+2. User account balance is lower than the bill amount.
+</t>
+  </si>
+  <si>
+    <t>Insert Card &gt; Select Language &gt; Enter valid PIN &gt; Select Bill Payment &gt; Select SLIC &gt; Select General Insurance &gt; Enter Customer Reference Number &gt; Enter Amount &gt; Select Account with low balance &gt; Confirm Bill Payment</t>
+  </si>
+  <si>
+    <t>Transaction is declined, an "Insufficient Funds" error message is displayed, and no receipt is printed.</t>
+  </si>
 </sst>
 </file>
 
@@ -2562,7 +2824,7 @@
   <numFmts count="1">
     <numFmt numFmtId="0" formatCode="General"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -2632,6 +2894,16 @@
       <sz val="13"/>
       <color indexed="8"/>
       <name val="Times New Roman"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color indexed="8"/>
+      <name val="Times Roman"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <color indexed="8"/>
+      <name val="Helvetica Neue"/>
     </font>
   </fonts>
   <fills count="9">
@@ -2928,7 +3200,7 @@
       <alignment vertical="bottom"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="114">
+  <cellXfs count="123">
     <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -3266,6 +3538,33 @@
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="9" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="49" fontId="13" fillId="4" borderId="14" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="13" fillId="4" borderId="14" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="4" borderId="14" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
@@ -4664,6 +4963,102 @@
         <v>28</v>
       </c>
     </row>
+    <row r="35">
+      <c r="B35" t="s" s="3">
+        <v>764</v>
+      </c>
+      <c r="C35" s="3"/>
+      <c r="D35" s="3"/>
+    </row>
+    <row r="36">
+      <c r="B36" s="4"/>
+      <c r="C36" t="s" s="4">
+        <v>5</v>
+      </c>
+      <c r="D36" t="s" s="5">
+        <v>765</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" t="s" s="3">
+        <v>778</v>
+      </c>
+      <c r="C37" s="3"/>
+      <c r="D37" s="3"/>
+    </row>
+    <row r="38">
+      <c r="B38" s="4"/>
+      <c r="C38" t="s" s="4">
+        <v>5</v>
+      </c>
+      <c r="D38" t="s" s="5">
+        <v>779</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" t="s" s="3">
+        <v>800</v>
+      </c>
+      <c r="C39" s="3"/>
+      <c r="D39" s="3"/>
+    </row>
+    <row r="40">
+      <c r="B40" s="4"/>
+      <c r="C40" t="s" s="4">
+        <v>5</v>
+      </c>
+      <c r="D40" t="s" s="5">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" t="s" s="3">
+        <v>808</v>
+      </c>
+      <c r="C41" s="3"/>
+      <c r="D41" s="3"/>
+    </row>
+    <row r="42">
+      <c r="B42" s="4"/>
+      <c r="C42" t="s" s="4">
+        <v>5</v>
+      </c>
+      <c r="D42" t="s" s="5">
+        <v>808</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" t="s" s="3">
+        <v>822</v>
+      </c>
+      <c r="C43" s="3"/>
+      <c r="D43" s="3"/>
+    </row>
+    <row r="44">
+      <c r="B44" s="4"/>
+      <c r="C44" t="s" s="4">
+        <v>5</v>
+      </c>
+      <c r="D44" t="s" s="5">
+        <v>822</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" t="s" s="3">
+        <v>830</v>
+      </c>
+      <c r="C45" s="3"/>
+      <c r="D45" s="3"/>
+    </row>
+    <row r="46">
+      <c r="B46" s="4"/>
+      <c r="C46" t="s" s="4">
+        <v>5</v>
+      </c>
+      <c r="D46" t="s" s="5">
+        <v>830</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B3:D3"/>
@@ -4695,6 +5090,12 @@
     <hyperlink ref="D30" location="'Admin _ Supervisor Functions-Ne'!R1C1" tooltip="" display="Admin _ Supervisor Functions-Ne"/>
     <hyperlink ref="D32" location="'Credit_Card_Positive_Scenario'!R1C1" tooltip="" display="Credit_Card_Positive_Scenario"/>
     <hyperlink ref="D34" location="'Credit_Card_Negative_Scenario'!R1C1" tooltip="" display="Credit_Card_Negative_Scenario"/>
+    <hyperlink ref="D36" location="'Other_Bank_Card_Positive_Scenar'!R1C1" tooltip="" display="Other_Bank_Card_Positive_Scenar"/>
+    <hyperlink ref="D38" location="'Other_Bank_Card_Negative_Scenar'!R1C1" tooltip="" display="Other_Bank_Card_Negative_Scenar"/>
+    <hyperlink ref="D40" location="'SLIC Life Positive'!R1C1" tooltip="" display="SLIC Life Positive"/>
+    <hyperlink ref="D42" location="'SLIC Life Negative'!R1C1" tooltip="" display="SLIC Life Negative"/>
+    <hyperlink ref="D44" location="'SLIC General Positive'!R1C1" tooltip="" display="SLIC General Positive"/>
+    <hyperlink ref="D46" location="'SLIC General Negative'!R1C1" tooltip="" display="SLIC General Negative"/>
   </hyperlinks>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
   <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
@@ -4845,7 +5246,7 @@
       <c r="M4" s="85"/>
       <c r="N4" s="56"/>
     </row>
-    <row r="5" ht="30" customHeight="1">
+    <row r="5" ht="39.1" customHeight="1">
       <c r="A5" t="s" s="33">
         <v>621</v>
       </c>
@@ -6012,6 +6413,978 @@
       <c r="L10" s="111"/>
       <c r="M10" s="111"/>
       <c r="N10" s="112"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
+  <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
+  <headerFooter>
+    <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:N6"/>
+  <sheetFormatPr defaultColWidth="15.3333" defaultRowHeight="15.4" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col min="1" max="1" width="25.0703" style="114" customWidth="1"/>
+    <col min="2" max="2" width="18.5" style="114" customWidth="1"/>
+    <col min="3" max="3" width="30.5" style="114" customWidth="1"/>
+    <col min="4" max="4" width="32.6719" style="114" customWidth="1"/>
+    <col min="5" max="5" width="45.6719" style="114" customWidth="1"/>
+    <col min="6" max="6" width="46.1719" style="114" customWidth="1"/>
+    <col min="7" max="7" width="36.6719" style="114" customWidth="1"/>
+    <col min="8" max="8" width="15.3516" style="114" customWidth="1"/>
+    <col min="9" max="9" width="27.6719" style="114" customWidth="1"/>
+    <col min="10" max="10" width="14.5" style="114" customWidth="1"/>
+    <col min="11" max="13" width="15.3516" style="114" customWidth="1"/>
+    <col min="14" max="14" width="29.5" style="114" customWidth="1"/>
+    <col min="15" max="16384" width="15.3516" style="114" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="18" customHeight="1">
+      <c r="A1" t="s" s="45">
+        <v>766</v>
+      </c>
+      <c r="B1" s="46"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
+      <c r="G1" s="47"/>
+      <c r="H1" s="47"/>
+      <c r="I1" s="47"/>
+      <c r="J1" s="47"/>
+      <c r="K1" s="47"/>
+      <c r="L1" s="47"/>
+      <c r="M1" s="47"/>
+      <c r="N1" s="47"/>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" t="s" s="48">
+        <v>32</v>
+      </c>
+      <c r="B2" t="s" s="48">
+        <v>33</v>
+      </c>
+      <c r="C2" t="s" s="48">
+        <v>34</v>
+      </c>
+      <c r="D2" t="s" s="48">
+        <v>35</v>
+      </c>
+      <c r="E2" t="s" s="48">
+        <v>36</v>
+      </c>
+      <c r="F2" t="s" s="48">
+        <v>37</v>
+      </c>
+      <c r="G2" t="s" s="48">
+        <v>38</v>
+      </c>
+      <c r="H2" t="s" s="75">
+        <v>39</v>
+      </c>
+      <c r="I2" t="s" s="75">
+        <v>40</v>
+      </c>
+      <c r="J2" t="s" s="75">
+        <v>370</v>
+      </c>
+      <c r="K2" t="s" s="48">
+        <v>369</v>
+      </c>
+      <c r="L2" t="s" s="48">
+        <v>42</v>
+      </c>
+      <c r="M2" t="s" s="48">
+        <v>43</v>
+      </c>
+      <c r="N2" t="s" s="48">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="3" ht="93.85" customHeight="1">
+      <c r="A3" t="s" s="33">
+        <v>767</v>
+      </c>
+      <c r="B3" t="s" s="50">
+        <v>768</v>
+      </c>
+      <c r="C3" t="s" s="82">
+        <v>769</v>
+      </c>
+      <c r="D3" t="s" s="82">
+        <v>770</v>
+      </c>
+      <c r="E3" t="s" s="98">
+        <v>488</v>
+      </c>
+      <c r="F3" t="s" s="98">
+        <v>771</v>
+      </c>
+      <c r="G3" s="91"/>
+      <c r="H3" s="91"/>
+      <c r="I3" s="91"/>
+      <c r="J3" s="91"/>
+      <c r="K3" s="91"/>
+      <c r="L3" s="85"/>
+      <c r="M3" s="85"/>
+      <c r="N3" s="56"/>
+    </row>
+    <row r="4" ht="82.4" customHeight="1">
+      <c r="A4" t="s" s="33">
+        <v>772</v>
+      </c>
+      <c r="B4" t="s" s="50">
+        <v>773</v>
+      </c>
+      <c r="C4" t="s" s="82">
+        <v>774</v>
+      </c>
+      <c r="D4" t="s" s="82">
+        <v>775</v>
+      </c>
+      <c r="E4" t="s" s="98">
+        <v>776</v>
+      </c>
+      <c r="F4" t="s" s="98">
+        <v>777</v>
+      </c>
+      <c r="G4" s="91"/>
+      <c r="H4" s="91"/>
+      <c r="I4" s="91"/>
+      <c r="J4" s="91"/>
+      <c r="K4" s="91"/>
+      <c r="L4" s="85"/>
+      <c r="M4" s="85"/>
+      <c r="N4" s="56"/>
+    </row>
+    <row r="5" ht="14.5" customHeight="1">
+      <c r="A5" s="103"/>
+      <c r="B5" s="105"/>
+      <c r="C5" s="105"/>
+      <c r="D5" s="105"/>
+      <c r="E5" s="105"/>
+      <c r="F5" s="105"/>
+      <c r="G5" s="105"/>
+      <c r="H5" s="105"/>
+      <c r="I5" s="105"/>
+      <c r="J5" s="105"/>
+      <c r="K5" s="105"/>
+      <c r="L5" s="105"/>
+      <c r="M5" s="105"/>
+      <c r="N5" s="106"/>
+    </row>
+    <row r="6" ht="14.5" customHeight="1">
+      <c r="A6" s="110"/>
+      <c r="B6" s="111"/>
+      <c r="C6" s="111"/>
+      <c r="D6" s="111"/>
+      <c r="E6" s="111"/>
+      <c r="F6" s="111"/>
+      <c r="G6" s="111"/>
+      <c r="H6" s="111"/>
+      <c r="I6" s="111"/>
+      <c r="J6" s="111"/>
+      <c r="K6" s="111"/>
+      <c r="L6" s="111"/>
+      <c r="M6" s="111"/>
+      <c r="N6" s="112"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
+  <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
+  <headerFooter>
+    <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:N8"/>
+  <sheetFormatPr defaultColWidth="15.3333" defaultRowHeight="15.4" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col min="1" max="1" width="25.0703" style="115" customWidth="1"/>
+    <col min="2" max="2" width="18.5" style="115" customWidth="1"/>
+    <col min="3" max="3" width="30.5" style="115" customWidth="1"/>
+    <col min="4" max="4" width="32.6719" style="115" customWidth="1"/>
+    <col min="5" max="5" width="45.6719" style="115" customWidth="1"/>
+    <col min="6" max="6" width="46.1719" style="115" customWidth="1"/>
+    <col min="7" max="7" width="36.6719" style="115" customWidth="1"/>
+    <col min="8" max="8" width="15.3516" style="115" customWidth="1"/>
+    <col min="9" max="9" width="27.6719" style="115" customWidth="1"/>
+    <col min="10" max="10" width="14.5" style="115" customWidth="1"/>
+    <col min="11" max="13" width="15.3516" style="115" customWidth="1"/>
+    <col min="14" max="14" width="29.5" style="115" customWidth="1"/>
+    <col min="15" max="16384" width="15.3516" style="115" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="18" customHeight="1">
+      <c r="A1" t="s" s="72">
+        <v>780</v>
+      </c>
+      <c r="B1" s="73"/>
+      <c r="C1" s="73"/>
+      <c r="D1" s="73"/>
+      <c r="E1" s="73"/>
+      <c r="F1" s="73"/>
+      <c r="G1" s="73"/>
+      <c r="H1" s="73"/>
+      <c r="I1" s="73"/>
+      <c r="J1" s="73"/>
+      <c r="K1" s="73"/>
+      <c r="L1" s="73"/>
+      <c r="M1" s="73"/>
+      <c r="N1" s="73"/>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" t="s" s="48">
+        <v>32</v>
+      </c>
+      <c r="B2" t="s" s="48">
+        <v>33</v>
+      </c>
+      <c r="C2" t="s" s="48">
+        <v>34</v>
+      </c>
+      <c r="D2" t="s" s="48">
+        <v>35</v>
+      </c>
+      <c r="E2" t="s" s="48">
+        <v>36</v>
+      </c>
+      <c r="F2" t="s" s="48">
+        <v>37</v>
+      </c>
+      <c r="G2" t="s" s="48">
+        <v>38</v>
+      </c>
+      <c r="H2" t="s" s="75">
+        <v>39</v>
+      </c>
+      <c r="I2" t="s" s="75">
+        <v>40</v>
+      </c>
+      <c r="J2" t="s" s="75">
+        <v>370</v>
+      </c>
+      <c r="K2" t="s" s="48">
+        <v>369</v>
+      </c>
+      <c r="L2" t="s" s="48">
+        <v>42</v>
+      </c>
+      <c r="M2" t="s" s="48">
+        <v>43</v>
+      </c>
+      <c r="N2" t="s" s="48">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="3" ht="93.85" customHeight="1">
+      <c r="A3" t="s" s="33">
+        <v>781</v>
+      </c>
+      <c r="B3" t="s" s="116">
+        <v>782</v>
+      </c>
+      <c r="C3" t="s" s="117">
+        <v>783</v>
+      </c>
+      <c r="D3" t="s" s="82">
+        <v>784</v>
+      </c>
+      <c r="E3" t="s" s="117">
+        <v>785</v>
+      </c>
+      <c r="F3" t="s" s="98">
+        <v>786</v>
+      </c>
+      <c r="G3" s="91"/>
+      <c r="H3" s="91"/>
+      <c r="I3" s="91"/>
+      <c r="J3" s="91"/>
+      <c r="K3" s="91"/>
+      <c r="L3" s="85"/>
+      <c r="M3" s="85"/>
+      <c r="N3" s="56"/>
+    </row>
+    <row r="4" ht="59.05" customHeight="1">
+      <c r="A4" t="s" s="33">
+        <v>787</v>
+      </c>
+      <c r="B4" t="s" s="50">
+        <v>788</v>
+      </c>
+      <c r="C4" t="s" s="82">
+        <v>789</v>
+      </c>
+      <c r="D4" t="s" s="82">
+        <v>790</v>
+      </c>
+      <c r="E4" t="s" s="98">
+        <v>791</v>
+      </c>
+      <c r="F4" t="s" s="98">
+        <v>792</v>
+      </c>
+      <c r="G4" s="91"/>
+      <c r="H4" s="91"/>
+      <c r="I4" s="91"/>
+      <c r="J4" s="91"/>
+      <c r="K4" s="91"/>
+      <c r="L4" s="85"/>
+      <c r="M4" s="85"/>
+      <c r="N4" s="56"/>
+    </row>
+    <row r="5" ht="50.4" customHeight="1">
+      <c r="A5" t="s" s="33">
+        <v>793</v>
+      </c>
+      <c r="B5" t="s" s="50">
+        <v>794</v>
+      </c>
+      <c r="C5" t="s" s="82">
+        <v>795</v>
+      </c>
+      <c r="D5" t="s" s="82">
+        <v>796</v>
+      </c>
+      <c r="E5" t="s" s="98">
+        <v>797</v>
+      </c>
+      <c r="F5" t="s" s="98">
+        <v>798</v>
+      </c>
+      <c r="G5" s="91"/>
+      <c r="H5" s="91"/>
+      <c r="I5" s="91"/>
+      <c r="J5" s="91"/>
+      <c r="K5" s="91"/>
+      <c r="L5" s="85"/>
+      <c r="M5" s="85"/>
+      <c r="N5" s="56"/>
+    </row>
+    <row r="6" ht="18.4" customHeight="1">
+      <c r="A6" t="s" s="33">
+        <v>799</v>
+      </c>
+      <c r="B6" s="50"/>
+      <c r="C6" s="82"/>
+      <c r="D6" s="82"/>
+      <c r="E6" s="98"/>
+      <c r="F6" s="98"/>
+      <c r="G6" s="91"/>
+      <c r="H6" s="91"/>
+      <c r="I6" s="91"/>
+      <c r="J6" s="91"/>
+      <c r="K6" s="91"/>
+      <c r="L6" s="85"/>
+      <c r="M6" s="85"/>
+      <c r="N6" s="56"/>
+    </row>
+    <row r="7" ht="14.5" customHeight="1">
+      <c r="A7" s="41"/>
+      <c r="B7" s="41"/>
+      <c r="C7" s="41"/>
+      <c r="D7" s="41"/>
+      <c r="E7" s="41"/>
+      <c r="F7" s="41"/>
+      <c r="G7" s="41"/>
+      <c r="H7" s="41"/>
+      <c r="I7" s="41"/>
+      <c r="J7" s="41"/>
+      <c r="K7" s="41"/>
+      <c r="L7" s="41"/>
+      <c r="M7" s="41"/>
+      <c r="N7" s="41"/>
+    </row>
+    <row r="8" ht="14.5" customHeight="1">
+      <c r="A8" s="41"/>
+      <c r="B8" s="41"/>
+      <c r="C8" s="41"/>
+      <c r="D8" s="41"/>
+      <c r="E8" s="41"/>
+      <c r="F8" s="41"/>
+      <c r="G8" s="41"/>
+      <c r="H8" s="41"/>
+      <c r="I8" s="41"/>
+      <c r="J8" s="41"/>
+      <c r="K8" s="41"/>
+      <c r="L8" s="41"/>
+      <c r="M8" s="41"/>
+      <c r="N8" s="41"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
+  <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
+  <headerFooter>
+    <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:N3"/>
+  <sheetFormatPr defaultColWidth="15.3333" defaultRowHeight="15.4" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col min="1" max="1" width="25.0703" style="118" customWidth="1"/>
+    <col min="2" max="2" width="18.5" style="118" customWidth="1"/>
+    <col min="3" max="3" width="30.5" style="118" customWidth="1"/>
+    <col min="4" max="4" width="32.6719" style="118" customWidth="1"/>
+    <col min="5" max="5" width="45.6719" style="118" customWidth="1"/>
+    <col min="6" max="6" width="46.1719" style="118" customWidth="1"/>
+    <col min="7" max="7" width="36.6719" style="118" customWidth="1"/>
+    <col min="8" max="8" width="15.3516" style="118" customWidth="1"/>
+    <col min="9" max="9" width="27.6719" style="118" customWidth="1"/>
+    <col min="10" max="10" width="14.5" style="118" customWidth="1"/>
+    <col min="11" max="13" width="15.3516" style="118" customWidth="1"/>
+    <col min="14" max="14" width="29.5" style="118" customWidth="1"/>
+    <col min="15" max="16384" width="15.3516" style="118" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="18" customHeight="1">
+      <c r="A1" t="s" s="72">
+        <v>801</v>
+      </c>
+      <c r="B1" s="73"/>
+      <c r="C1" s="73"/>
+      <c r="D1" s="73"/>
+      <c r="E1" s="73"/>
+      <c r="F1" s="73"/>
+      <c r="G1" s="73"/>
+      <c r="H1" s="73"/>
+      <c r="I1" s="73"/>
+      <c r="J1" s="73"/>
+      <c r="K1" s="73"/>
+      <c r="L1" s="73"/>
+      <c r="M1" s="73"/>
+      <c r="N1" s="73"/>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" t="s" s="48">
+        <v>32</v>
+      </c>
+      <c r="B2" t="s" s="48">
+        <v>33</v>
+      </c>
+      <c r="C2" t="s" s="48">
+        <v>34</v>
+      </c>
+      <c r="D2" t="s" s="48">
+        <v>35</v>
+      </c>
+      <c r="E2" t="s" s="48">
+        <v>36</v>
+      </c>
+      <c r="F2" t="s" s="48">
+        <v>37</v>
+      </c>
+      <c r="G2" t="s" s="48">
+        <v>38</v>
+      </c>
+      <c r="H2" t="s" s="75">
+        <v>39</v>
+      </c>
+      <c r="I2" t="s" s="75">
+        <v>40</v>
+      </c>
+      <c r="J2" t="s" s="75">
+        <v>370</v>
+      </c>
+      <c r="K2" t="s" s="48">
+        <v>369</v>
+      </c>
+      <c r="L2" t="s" s="48">
+        <v>42</v>
+      </c>
+      <c r="M2" t="s" s="48">
+        <v>43</v>
+      </c>
+      <c r="N2" t="s" s="48">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="3" ht="93.85" customHeight="1">
+      <c r="A3" t="s" s="33">
+        <v>802</v>
+      </c>
+      <c r="B3" t="s" s="116">
+        <v>803</v>
+      </c>
+      <c r="C3" t="s" s="117">
+        <v>804</v>
+      </c>
+      <c r="D3" t="s" s="119">
+        <v>805</v>
+      </c>
+      <c r="E3" t="s" s="117">
+        <v>806</v>
+      </c>
+      <c r="F3" t="s" s="98">
+        <v>807</v>
+      </c>
+      <c r="G3" s="91"/>
+      <c r="H3" s="91"/>
+      <c r="I3" s="91"/>
+      <c r="J3" s="91"/>
+      <c r="K3" s="91"/>
+      <c r="L3" s="85"/>
+      <c r="M3" s="85"/>
+      <c r="N3" s="56"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
+  <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
+  <headerFooter>
+    <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:N4"/>
+  <sheetFormatPr defaultColWidth="15.3333" defaultRowHeight="15.4" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col min="1" max="1" width="25.0703" style="120" customWidth="1"/>
+    <col min="2" max="2" width="18.5" style="120" customWidth="1"/>
+    <col min="3" max="3" width="30.5" style="120" customWidth="1"/>
+    <col min="4" max="4" width="32.6719" style="120" customWidth="1"/>
+    <col min="5" max="5" width="45.6719" style="120" customWidth="1"/>
+    <col min="6" max="6" width="46.1719" style="120" customWidth="1"/>
+    <col min="7" max="7" width="36.6719" style="120" customWidth="1"/>
+    <col min="8" max="8" width="15.3516" style="120" customWidth="1"/>
+    <col min="9" max="9" width="27.6719" style="120" customWidth="1"/>
+    <col min="10" max="10" width="14.5" style="120" customWidth="1"/>
+    <col min="11" max="13" width="15.3516" style="120" customWidth="1"/>
+    <col min="14" max="14" width="29.5" style="120" customWidth="1"/>
+    <col min="15" max="16384" width="15.3516" style="120" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="18" customHeight="1">
+      <c r="A1" t="s" s="72">
+        <v>809</v>
+      </c>
+      <c r="B1" s="73"/>
+      <c r="C1" s="73"/>
+      <c r="D1" s="73"/>
+      <c r="E1" s="73"/>
+      <c r="F1" s="73"/>
+      <c r="G1" s="73"/>
+      <c r="H1" s="73"/>
+      <c r="I1" s="73"/>
+      <c r="J1" s="73"/>
+      <c r="K1" s="73"/>
+      <c r="L1" s="73"/>
+      <c r="M1" s="73"/>
+      <c r="N1" s="73"/>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" t="s" s="48">
+        <v>32</v>
+      </c>
+      <c r="B2" t="s" s="48">
+        <v>33</v>
+      </c>
+      <c r="C2" t="s" s="48">
+        <v>34</v>
+      </c>
+      <c r="D2" t="s" s="48">
+        <v>35</v>
+      </c>
+      <c r="E2" t="s" s="48">
+        <v>36</v>
+      </c>
+      <c r="F2" t="s" s="48">
+        <v>37</v>
+      </c>
+      <c r="G2" t="s" s="48">
+        <v>38</v>
+      </c>
+      <c r="H2" t="s" s="75">
+        <v>39</v>
+      </c>
+      <c r="I2" t="s" s="75">
+        <v>40</v>
+      </c>
+      <c r="J2" t="s" s="75">
+        <v>370</v>
+      </c>
+      <c r="K2" t="s" s="48">
+        <v>369</v>
+      </c>
+      <c r="L2" t="s" s="48">
+        <v>42</v>
+      </c>
+      <c r="M2" t="s" s="48">
+        <v>43</v>
+      </c>
+      <c r="N2" t="s" s="48">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="3" ht="93.85" customHeight="1">
+      <c r="A3" t="s" s="33">
+        <v>810</v>
+      </c>
+      <c r="B3" t="s" s="116">
+        <v>811</v>
+      </c>
+      <c r="C3" t="s" s="117">
+        <v>812</v>
+      </c>
+      <c r="D3" t="s" s="119">
+        <v>813</v>
+      </c>
+      <c r="E3" t="s" s="117">
+        <v>814</v>
+      </c>
+      <c r="F3" t="s" s="98">
+        <v>815</v>
+      </c>
+      <c r="G3" s="91"/>
+      <c r="H3" s="91"/>
+      <c r="I3" s="91"/>
+      <c r="J3" s="91"/>
+      <c r="K3" s="91"/>
+      <c r="L3" s="85"/>
+      <c r="M3" s="85"/>
+      <c r="N3" s="56"/>
+    </row>
+    <row r="4" ht="93.85" customHeight="1">
+      <c r="A4" t="s" s="33">
+        <v>816</v>
+      </c>
+      <c r="B4" t="s" s="116">
+        <v>817</v>
+      </c>
+      <c r="C4" t="s" s="117">
+        <v>818</v>
+      </c>
+      <c r="D4" t="s" s="119">
+        <v>819</v>
+      </c>
+      <c r="E4" t="s" s="117">
+        <v>820</v>
+      </c>
+      <c r="F4" t="s" s="98">
+        <v>821</v>
+      </c>
+      <c r="G4" s="91"/>
+      <c r="H4" s="91"/>
+      <c r="I4" s="91"/>
+      <c r="J4" s="91"/>
+      <c r="K4" s="91"/>
+      <c r="L4" s="85"/>
+      <c r="M4" s="85"/>
+      <c r="N4" s="56"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
+  <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
+  <headerFooter>
+    <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:N3"/>
+  <sheetFormatPr defaultColWidth="15.3333" defaultRowHeight="15.4" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col min="1" max="1" width="25.0703" style="121" customWidth="1"/>
+    <col min="2" max="2" width="18.5" style="121" customWidth="1"/>
+    <col min="3" max="3" width="30.5" style="121" customWidth="1"/>
+    <col min="4" max="4" width="32.6719" style="121" customWidth="1"/>
+    <col min="5" max="5" width="45.6719" style="121" customWidth="1"/>
+    <col min="6" max="6" width="46.1719" style="121" customWidth="1"/>
+    <col min="7" max="7" width="36.6719" style="121" customWidth="1"/>
+    <col min="8" max="8" width="15.3516" style="121" customWidth="1"/>
+    <col min="9" max="9" width="27.6719" style="121" customWidth="1"/>
+    <col min="10" max="10" width="14.5" style="121" customWidth="1"/>
+    <col min="11" max="13" width="15.3516" style="121" customWidth="1"/>
+    <col min="14" max="14" width="29.5" style="121" customWidth="1"/>
+    <col min="15" max="16384" width="15.3516" style="121" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="18" customHeight="1">
+      <c r="A1" t="s" s="72">
+        <v>823</v>
+      </c>
+      <c r="B1" s="73"/>
+      <c r="C1" s="73"/>
+      <c r="D1" s="73"/>
+      <c r="E1" s="73"/>
+      <c r="F1" s="73"/>
+      <c r="G1" s="73"/>
+      <c r="H1" s="73"/>
+      <c r="I1" s="73"/>
+      <c r="J1" s="73"/>
+      <c r="K1" s="73"/>
+      <c r="L1" s="73"/>
+      <c r="M1" s="73"/>
+      <c r="N1" s="73"/>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" t="s" s="48">
+        <v>32</v>
+      </c>
+      <c r="B2" t="s" s="48">
+        <v>33</v>
+      </c>
+      <c r="C2" t="s" s="48">
+        <v>34</v>
+      </c>
+      <c r="D2" t="s" s="48">
+        <v>35</v>
+      </c>
+      <c r="E2" t="s" s="48">
+        <v>36</v>
+      </c>
+      <c r="F2" t="s" s="48">
+        <v>37</v>
+      </c>
+      <c r="G2" t="s" s="48">
+        <v>38</v>
+      </c>
+      <c r="H2" t="s" s="75">
+        <v>39</v>
+      </c>
+      <c r="I2" t="s" s="75">
+        <v>40</v>
+      </c>
+      <c r="J2" t="s" s="75">
+        <v>370</v>
+      </c>
+      <c r="K2" t="s" s="48">
+        <v>369</v>
+      </c>
+      <c r="L2" t="s" s="48">
+        <v>42</v>
+      </c>
+      <c r="M2" t="s" s="48">
+        <v>43</v>
+      </c>
+      <c r="N2" t="s" s="48">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="3" ht="93.85" customHeight="1">
+      <c r="A3" t="s" s="33">
+        <v>824</v>
+      </c>
+      <c r="B3" t="s" s="116">
+        <v>825</v>
+      </c>
+      <c r="C3" t="s" s="117">
+        <v>826</v>
+      </c>
+      <c r="D3" t="s" s="119">
+        <v>827</v>
+      </c>
+      <c r="E3" t="s" s="117">
+        <v>828</v>
+      </c>
+      <c r="F3" t="s" s="98">
+        <v>829</v>
+      </c>
+      <c r="G3" s="91"/>
+      <c r="H3" s="91"/>
+      <c r="I3" s="91"/>
+      <c r="J3" s="91"/>
+      <c r="K3" s="91"/>
+      <c r="L3" s="85"/>
+      <c r="M3" s="85"/>
+      <c r="N3" s="56"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
+  <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
+  <headerFooter>
+    <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:N4"/>
+  <sheetFormatPr defaultColWidth="15.3333" defaultRowHeight="15.4" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col min="1" max="1" width="25.0703" style="122" customWidth="1"/>
+    <col min="2" max="2" width="18.5" style="122" customWidth="1"/>
+    <col min="3" max="3" width="30.5" style="122" customWidth="1"/>
+    <col min="4" max="4" width="32.6719" style="122" customWidth="1"/>
+    <col min="5" max="5" width="45.6719" style="122" customWidth="1"/>
+    <col min="6" max="6" width="46.1719" style="122" customWidth="1"/>
+    <col min="7" max="7" width="36.6719" style="122" customWidth="1"/>
+    <col min="8" max="8" width="15.3516" style="122" customWidth="1"/>
+    <col min="9" max="9" width="27.6719" style="122" customWidth="1"/>
+    <col min="10" max="10" width="14.5" style="122" customWidth="1"/>
+    <col min="11" max="13" width="15.3516" style="122" customWidth="1"/>
+    <col min="14" max="14" width="29.5" style="122" customWidth="1"/>
+    <col min="15" max="16384" width="15.3516" style="122" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="18" customHeight="1">
+      <c r="A1" t="s" s="72">
+        <v>831</v>
+      </c>
+      <c r="B1" s="73"/>
+      <c r="C1" s="73"/>
+      <c r="D1" s="73"/>
+      <c r="E1" s="73"/>
+      <c r="F1" s="73"/>
+      <c r="G1" s="73"/>
+      <c r="H1" s="73"/>
+      <c r="I1" s="73"/>
+      <c r="J1" s="73"/>
+      <c r="K1" s="73"/>
+      <c r="L1" s="73"/>
+      <c r="M1" s="73"/>
+      <c r="N1" s="73"/>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" t="s" s="48">
+        <v>32</v>
+      </c>
+      <c r="B2" t="s" s="48">
+        <v>33</v>
+      </c>
+      <c r="C2" t="s" s="48">
+        <v>34</v>
+      </c>
+      <c r="D2" t="s" s="48">
+        <v>35</v>
+      </c>
+      <c r="E2" t="s" s="48">
+        <v>36</v>
+      </c>
+      <c r="F2" t="s" s="48">
+        <v>37</v>
+      </c>
+      <c r="G2" t="s" s="48">
+        <v>38</v>
+      </c>
+      <c r="H2" t="s" s="75">
+        <v>39</v>
+      </c>
+      <c r="I2" t="s" s="75">
+        <v>40</v>
+      </c>
+      <c r="J2" t="s" s="75">
+        <v>370</v>
+      </c>
+      <c r="K2" t="s" s="48">
+        <v>369</v>
+      </c>
+      <c r="L2" t="s" s="48">
+        <v>42</v>
+      </c>
+      <c r="M2" t="s" s="48">
+        <v>43</v>
+      </c>
+      <c r="N2" t="s" s="48">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="3" ht="93.85" customHeight="1">
+      <c r="A3" t="s" s="33">
+        <v>832</v>
+      </c>
+      <c r="B3" t="s" s="116">
+        <v>833</v>
+      </c>
+      <c r="C3" t="s" s="117">
+        <v>834</v>
+      </c>
+      <c r="D3" t="s" s="119">
+        <v>813</v>
+      </c>
+      <c r="E3" t="s" s="117">
+        <v>835</v>
+      </c>
+      <c r="F3" t="s" s="98">
+        <v>836</v>
+      </c>
+      <c r="G3" s="91"/>
+      <c r="H3" s="91"/>
+      <c r="I3" s="91"/>
+      <c r="J3" s="91"/>
+      <c r="K3" s="91"/>
+      <c r="L3" s="85"/>
+      <c r="M3" s="85"/>
+      <c r="N3" s="56"/>
+    </row>
+    <row r="4" ht="93.85" customHeight="1">
+      <c r="A4" t="s" s="33">
+        <v>837</v>
+      </c>
+      <c r="B4" t="s" s="116">
+        <v>838</v>
+      </c>
+      <c r="C4" t="s" s="117">
+        <v>839</v>
+      </c>
+      <c r="D4" t="s" s="119">
+        <v>840</v>
+      </c>
+      <c r="E4" t="s" s="117">
+        <v>841</v>
+      </c>
+      <c r="F4" t="s" s="98">
+        <v>842</v>
+      </c>
+      <c r="G4" s="91"/>
+      <c r="H4" s="91"/>
+      <c r="I4" s="91"/>
+      <c r="J4" s="91"/>
+      <c r="K4" s="91"/>
+      <c r="L4" s="85"/>
+      <c r="M4" s="85"/>
+      <c r="N4" s="56"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>